<commit_message>
Import Excel de reception : quantites en kilogrammes
- Le modele remplace la colonne quantite (unite de l'article, ambigue) par
  quantite_kg pour les matieres premieres et quantite_unites pour les
  articles de conditionnement ; prix et frais d'approche au kg (MP) ou a
  l'unite (AC).
- Conversion automatique vers l'unite de stock : g (x 1000), L et ml via la
  masse volumique de la fiche article (ligne rejetee si elle manque) ; le
  prix au kg est ramene a l'unite de stock.
- Rejets motives : MP saisie en unites, AC saisi en kg, deux quantites
  renseignees, nombre d'unites non entier, fichier de l'ancien modele.
- L'apercu affiche la quantite saisie et l'entree en stock convertie.
- Tests et parcours navigateur mis a jour (63 tests).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQJkoxKcYWHePrTa9oVJLg
</commit_message>
<xml_diff>
--- a/frontend/e2e/fixtures/reception.xlsx
+++ b/frontend/e2e/fixtures/reception.xlsx
@@ -12,12 +12,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>code_sku</t>
   </si>
   <si>
-    <t>quantite</t>
+    <t>quantite_kg</t>
+  </si>
+  <si>
+    <t>quantite_unites</t>
   </si>
   <si>
     <t>lot_fournisseur</t>
@@ -41,7 +44,10 @@
     <t>Code article (MP ou AC) (obligatoire)</t>
   </si>
   <si>
-    <t>Quantite recue, dans l'unite de l'article (obligatoire)</t>
+    <t>Quantite recue en kilogrammes (matiere premiere)</t>
+  </si>
+  <si>
+    <t>Nombre d'unites recues (article de conditionnement)</t>
   </si>
   <si>
     <t>Numero de lot fournisseur (obligatoire)</t>
@@ -50,10 +56,10 @@
     <t>DLUO ou peremption (JJ/MM/AAAA)</t>
   </si>
   <si>
-    <t>Prix achat unitaire HT (obligatoire)</t>
-  </si>
-  <si>
-    <t>Frais d'approche unitaires</t>
+    <t>Prix achat HT par kg (MP) ou par unite (AC) (obligatoire)</t>
+  </si>
+  <si>
+    <t>Frais d'approche par kg (MP) ou par unite (AC)</t>
   </si>
   <si>
     <t>Emplacement</t>
@@ -86,6 +92,12 @@
     <t>conforme</t>
   </si>
   <si>
+    <t>MP-HUJ-003</t>
+  </si>
+  <si>
+    <t>HUJ-E2E-01</t>
+  </si>
+  <si>
     <t>MP-INCONNU</t>
   </si>
   <si>
@@ -101,7 +113,10 @@
     <t>• Le code doit designer une matiere premiere ou un article de conditionnement existant et disponible.</t>
   </si>
   <si>
-    <t>• La quantite s'exprime dans l'unite de gestion de l'article (kg, g, L, ml ou U).</t>
+    <t>• Matiere premiere : quantite en kilogrammes (colonne quantite_kg) et prix par kg. Article de conditionnement : nombre d'unites (colonne quantite_unites) et prix par unite.</t>
+  </si>
+  <si>
+    <t>• Une matiere premiere geree en g, L ou ml est convertie a l'import (les volumes avec la masse volumique de sa fiche article).</t>
   </si>
   <si>
     <t>• Le certificat de conformite est facultatif : il se joint ensuite depuis la fiche de chaque lot.</t>
@@ -516,17 +531,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" customWidth="1"/>
-    <col min="5" max="8" width="16" customWidth="1"/>
+    <col min="1" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16" style="1" customWidth="1"/>
+    <col min="6" max="7" width="18" customWidth="1"/>
+    <col min="8" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -536,10 +551,10 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
@@ -551,98 +566,119 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" ht="42" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="E2" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="F2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>300</v>
       </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3">
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3">
         <v>36</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
       <c r="H3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4">
+        <v>23</v>
+      </c>
+      <c r="C4">
         <v>1500</v>
       </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4">
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4">
         <v>62</v>
       </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5">
+        <v>87</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5">
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur non autorisee" error="Valeurs possibles : quarantaine, conforme" sqref="H10:H1000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur non autorisee" error="Valeurs possibles : quarantaine, conforme" sqref="I10:I1000">
       <formula1>"quarantaine,conforme"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur non autorisee" error="Valeurs possibles : quarantaine, conforme" sqref="H3:H1000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur non autorisee" error="Valeurs possibles : quarantaine, conforme" sqref="I3:I1000">
       <formula1>"quarantaine,conforme"</formula1>
     </dataValidation>
   </dataValidations>
@@ -653,7 +689,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -661,32 +697,37 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>